<commit_message>
July 2, 2026 deck v2 — add Equity Savings VR category (8 peers, new in BirlaMFPR 30-Jun-26)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/July 2, 2026/Data/Mapping/Mapping VR to MFI names.xlsx
+++ b/July 2, 2026/Data/Mapping/Mapping VR to MFI names.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D583"/>
+  <dimension ref="A1:D592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12018,6 +12018,184 @@
         </is>
       </c>
       <c r="D583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Aditya Birla Sun Life Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B584" t="n">
+        <v>132995</v>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Aditya Birla Sun Life Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Axis Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B585" t="n">
+        <v>135120</v>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Axis Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Bandhan Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B586" t="n">
+        <v>118477</v>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Bandhan Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Edelweiss Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B587" t="n">
+        <v>140347</v>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Edelweiss Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Franklin India Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B588" t="n">
+        <v>144466</v>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Franklin India Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>ICICI Prudential Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B589" t="n">
+        <v>133054</v>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>ICICI Prudential Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Nippon India Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B590" t="n">
+        <v>134594</v>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Nippon India Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>PGIM India Equity Savings Fund - Direct Plan</t>
+        </is>
+      </c>
+      <c r="B591" t="n">
+        <v>138376</v>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>PGIM India Equity Savings Fund - Dir - Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>NIFTY Equity Savings Total Return Index</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>bench</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Equity Savings</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12030,7 +12208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12505,6 +12683,23 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>NIFTY Equity Savings Total Return Index</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Nifty Equity Savings TRI</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>VR Benchmarks NAV from MFI - July 2 2026.xlsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>